<commit_message>
Add service packages, checkout upsell, and multi-video hero
Implement PRD requirement 11: sell installation and demo packages as
regular products, with a robot selector on their detail page that ties
each service to a specific robot and carries that association through
the cart, checkout, and order record. Before payment, prompt a matching
installation/demo upsell sized to the robots in the cart; dismissing it
never blocks checkout.

Extend the hero to cycle through a playlist of background videos set in
data/siteConfig.ts, falling back to the animated lawn scene when none
are configured.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B52ED5E3-7BC7-4C97-86E6-6AE01E3EA252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{05C71A75-C9B6-48D9-9CED-00C31B9BE5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="3" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
+    <sheet name="DEFINITIONS" sheetId="2" r:id="rId2"/>
+    <sheet name="Useful resources" sheetId="3" r:id="rId3"/>
+    <sheet name="WebCredentials" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,9 +42,221 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="69">
+  <si>
+    <t>PROJECT REQUIREMENTS</t>
+  </si>
+  <si>
+    <t>PROJECT No:</t>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>FULL PROJECT NAME:</t>
+  </si>
+  <si>
+    <t>Ecommerce-RaasPal</t>
+  </si>
+  <si>
+    <t>DATE:</t>
+  </si>
+  <si>
+    <t>PROJECT MANAGER:</t>
+  </si>
+  <si>
+    <t>Swan Htet Aung (Branny)</t>
+  </si>
+  <si>
+    <t>REQUIREMENT LIST</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>REQUIREMENT DESCRIPTION</t>
+  </si>
+  <si>
+    <t>REQUESTED BY</t>
+  </si>
+  <si>
+    <t>CATEGORY</t>
+  </si>
+  <si>
+    <t>PRIORITY</t>
+  </si>
+  <si>
+    <t>ACCEPTANCE CRITERIA</t>
+  </si>
+  <si>
+    <t>Give each requirement a unique ID.</t>
+  </si>
+  <si>
+    <t>The feature, function, condition or capability that is required from the project, product, service or result.</t>
+  </si>
+  <si>
+    <t>The stakeholder who requested the requirement.</t>
+  </si>
+  <si>
+    <t>The category or grouping of the requirement for example: functional, technical, operational, KPI (result metric), transitional.</t>
+  </si>
+  <si>
+    <t>The priority of the requirement for example: P1, P2, P3 or MoSCoW (Must have, should have, could have, won't have).</t>
+  </si>
+  <si>
+    <t>The criteria that the requirement must have for it to be accepted by the project stakeholders.</t>
+  </si>
+  <si>
+    <t>Homepage – Hero Banner</t>
+  </si>
+  <si>
+    <t>Khun Pom</t>
+  </si>
+  <si>
+    <t>functional</t>
+  </si>
+  <si>
+    <t>Must have</t>
+  </si>
+  <si>
+    <t>Hero banner displays headline, subtext, and CTA buttons (Find Your Ideal Robot, Book a Free Demo) above the fold; plays uploaded video when one is attached; falls back to default animation/illustration automatically when no video is set; nav menu visible below.</t>
+  </si>
+  <si>
+    <t>Homepage – Trust / About Stats ("Who We Are")</t>
+  </si>
+  <si>
+    <t>Should have</t>
+  </si>
+  <si>
+    <t>Displays "WHO WE ARE" eyebrow text, heading, and short about paragraph; shows 4 stat cards (500+ Robots Deployed, 4.9★ Customer Rating, 10+ Service Locations, 30 Day Returns).</t>
+  </si>
+  <si>
+    <t>Homepage – Why Choose Us</t>
+  </si>
+  <si>
+    <t>เ</t>
+  </si>
+  <si>
+    <t>Homepage – Popular Products</t>
+  </si>
+  <si>
+    <t>Displays popular/featured product cards when scrolled down; each product is clickable and navigates to its product detail page.</t>
+  </si>
+  <si>
+    <t>Homepage – YouTube CTA Section</t>
+  </si>
+  <si>
+    <t>Could have</t>
+  </si>
+  <si>
+    <t>Displays play icon, heading "Subscribe to RoboStore TV", subtext, and "Subscribe on YouTube" button; button links to correct YouTube channel.</t>
+  </si>
+  <si>
+    <t>Homepage – Footer</t>
+  </si>
+  <si>
+    <t>Displays brand block (logo, tagline "Time for Life™", copyright, social icons), Policies column (Refunds and Returns, Privacy Policy, Terms and Conditions, Shipping, Payment and Finance Options, Warranty), About column (About Us, Contact, Support, Blog, Find My Robot), and payment/trust bar with payment method badges (PromptPay, Visa, Mastercard, Amex, Bank Transfer).</t>
+  </si>
+  <si>
+    <t>Shop / product listing pages</t>
+  </si>
+  <si>
+    <t>Product detail page</t>
+  </si>
+  <si>
+    <t>Thai/English translation (i18n)</t>
+  </si>
+  <si>
+    <t>technical</t>
+  </si>
+  <si>
+    <t>Cart + Checkout</t>
+  </si>
+  <si>
+    <t>TERM</t>
+  </si>
+  <si>
+    <t>DEFINITION</t>
+  </si>
+  <si>
+    <t>MoSCoW</t>
+  </si>
+  <si>
+    <t>A prioritization technique: Must have, Should have, Could have, Won't have.</t>
+  </si>
+  <si>
+    <t>KPI</t>
+  </si>
+  <si>
+    <t>Key Performance Indicator — a measurable value used to track a result.</t>
+  </si>
+  <si>
+    <t>P1/P2/P3</t>
+  </si>
+  <si>
+    <t>Priority ranking, where P1 is the highest priority.</t>
+  </si>
+  <si>
+    <t>RESOURCE</t>
+  </si>
+  <si>
+    <t>LINK / NOTES</t>
+  </si>
+  <si>
+    <t>Requirements gathering template</t>
+  </si>
+  <si>
+    <t>Add link here</t>
+  </si>
+  <si>
+    <t>Supabase DB</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>Raas1234@Pal</t>
+  </si>
+  <si>
+    <t>Admin Account</t>
+  </si>
+  <si>
+    <t>swan.h@raaspal.com</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>Checkout Upsell + Standalone Installation/Demo Packages</t>
+  </si>
+  <si>
+    <t>Installation Service and "Request a Demo" packages are listed as regular purchasable products on the Shop/product listing page (with their own product detail page, price, and "Add to Cart" button) so customers can buy them independently at any time. Additionally, before payment is submitted during checkout, the system prompts the customer with an upsell offer relevant to the products in their cart: (a) Installation Service packages tiered by coverage area/hours (e.g. Up to 1000m² / 2.5 hrs, 2000m² / 3.5 hrs, 10000m² / 8 hrs) matched to the robot(s) added, or (b) the "Request a Demo" package. Customer can add the selected package to the cart and continue, or dismiss the prompt and proceed to payment without it; dismissing does not block checkout.</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>This field describes whether the requirement is implemented or not.</t>
+  </si>
+  <si>
+    <t>Product Recommendation feature</t>
+  </si>
+  <si>
+    <t>Contact Sales</t>
+  </si>
+  <si>
+    <t>Request Quotation</t>
+  </si>
+  <si>
+    <t>Sokochan API  integration</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -48,16 +264,76 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F6FC5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,14 +341,78 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -86,6 +426,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -403,11 +760,893 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="408" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{06EE7FF3-6D25-4CC1-9A93-57B582D07718}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;67117232-04d2-44be-9b2d-3c224a7c80fd&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A72840-96E5-404A-A50D-490FFB57DF4F}">
-  <dimension ref="A1"/>
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="23.54296875" customWidth="1"/>
+    <col min="4" max="5" width="27.26953125" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+    <col min="7" max="7" width="14.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="16"/>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="17"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="18">
+        <v>46212</v>
+      </c>
+      <c r="C3" s="16"/>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="17"/>
+    </row>
+    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.4">
+      <c r="A5" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="12"/>
+    </row>
+    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="73" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="7">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>2</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7">
+        <v>3</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="7">
+        <v>4</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7">
+        <v>5</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7">
+        <v>6</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="5">
+        <v>7</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>8</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>9</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>10</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>11</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G18" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>12</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="6"/>
+      <c r="G19" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>13</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="6"/>
+      <c r="G20" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>14</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="6"/>
+      <c r="G21" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>15</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="6"/>
+      <c r="G22" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="E3:F3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D2344B6-7BC6-4AED-91CB-879E7DD96A50}">
+  <sheetPr>
+    <tabColor rgb="FF4472C4"/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="32.7265625" customWidth="1"/>
+    <col min="2" max="2" width="58.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC28DB7D-40EE-4F0F-8EB0-570A14F827B7}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="32.7265625" customWidth="1"/>
+    <col min="2" max="2" width="58.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E048D108-EE43-43FF-98E7-58D5322B5F5D}">
+  <dimension ref="A2:E4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="4" max="4" width="13.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" xr:uid="{30137649-3972-4052-B5A9-9F3C45EE7559}"/>
+    <hyperlink ref="E4" r:id="rId2" xr:uid="{FF521E3C-935E-4025-8514-AC05FDAFC578}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034E905B39333B74FA95898E771115485" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5aff7705dba03f1ca66de0bba948c32">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e484384a-471b-4d38-9bd4-f717a40f978d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a032af748e954b11f4b97a83e204a1c4" ns3:_="">
+    <xsd:import namespace="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e484384a-471b-4d38-9bd4-f717a40f978d" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceDateTaken" ma:index="8" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="12" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_activity" ma:index="13" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="14" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSystemTags" ma:index="15" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8FE9B93-FBF1-4A06-954E-D242AA736238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add product image URLs and Contact Sales page
Products (including service packages) can now use a custom photo URL
instead of the built-in illustration, editable from the admin form
with a live preview. Also adds /contact-sales (PRD req 19) with phone,
email, and a LINE QR slot, linked from the navbar's Contact dropdown.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05C71A75-C9B6-48D9-9CED-00C31B9BE5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{38C3A086-FF17-4FE8-82A3-FEE89E692334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="3" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <sheet name="WebCredentials" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="79">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -250,6 +249,36 @@
   </si>
   <si>
     <t>Sokochan API  integration</t>
+  </si>
+  <si>
+    <t>Contact sales features should include a line qr of the sales team</t>
+  </si>
+  <si>
+    <t>User profile page should contain the user's address, the details of the user.</t>
+  </si>
+  <si>
+    <t>User  Profile Page</t>
+  </si>
+  <si>
+    <t>User Details Editing feature</t>
+  </si>
+  <si>
+    <t>operational</t>
+  </si>
+  <si>
+    <t>User profile page will have a button to edit the user details</t>
+  </si>
+  <si>
+    <t>User details page will contain the addresses the user added to his/her profile and also the editing feature of the address.</t>
+  </si>
+  <si>
+    <t>User Address Details section</t>
+  </si>
+  <si>
+    <t>Contact Sales full function</t>
+  </si>
+  <si>
+    <t>User clicks contact sales button in the contact drop down at the nav bar and he should be led to a page that gives contact info about the sales team or line qr.</t>
   </si>
 </sst>
 </file>
@@ -443,6 +472,10 @@
     </a>
   </bag>
 </FeaturePropertyBags>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -792,7 +825,7 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -1132,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="257.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>11</v>
       </c>
@@ -1152,7 +1185,7 @@
         <v>62</v>
       </c>
       <c r="G18" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -1176,7 +1209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>13</v>
       </c>
@@ -1192,7 +1225,9 @@
       <c r="E20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="6"/>
+      <c r="F20" s="6" t="s">
+        <v>69</v>
+      </c>
       <c r="G20" s="11" t="b">
         <v>0</v>
       </c>
@@ -1239,36 +1274,791 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
+    <row r="23" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="5">
+        <v>16</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="6"/>
+      <c r="E23" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="G23" s="11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
+    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>17</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>72</v>
+      </c>
       <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="6"/>
+      <c r="D24" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="G24" s="11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
+    <row r="25" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="5">
+        <v>18</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="6"/>
+      <c r="D25" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>75</v>
+      </c>
       <c r="G25" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A26" s="5">
+        <v>19</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G26" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="5"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="6"/>
+      <c r="G47" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="6"/>
+      <c r="G49" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="6"/>
+      <c r="G51" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" s="5"/>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="6"/>
+      <c r="G62" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="6"/>
+      <c r="G65" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="5"/>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="6"/>
+      <c r="G71" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5"/>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="6"/>
+      <c r="G72" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="6"/>
+      <c r="G73" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" s="5"/>
+      <c r="B74" s="5"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="6"/>
+      <c r="G74" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" s="5"/>
+      <c r="B75" s="5"/>
+      <c r="C75" s="5"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="6"/>
+      <c r="G75" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" s="5"/>
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" s="5"/>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="6"/>
+      <c r="G77" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" s="5"/>
+      <c r="B78" s="5"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="6"/>
+      <c r="G78" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="6"/>
+      <c r="G79" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" s="5"/>
+      <c r="B80" s="5"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="6"/>
+      <c r="G80" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="6"/>
+      <c r="G81" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" s="5"/>
+      <c r="B82" s="5"/>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="6"/>
+      <c r="G82" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="6"/>
+      <c r="G83" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
+      <c r="C84" s="5"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="6"/>
+      <c r="G85" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A86" s="5"/>
+      <c r="B86" s="5"/>
+      <c r="C86" s="5"/>
+      <c r="D86" s="5"/>
+      <c r="E86" s="5"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" s="5"/>
+      <c r="B87" s="5"/>
+      <c r="C87" s="5"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="5"/>
+      <c r="F87" s="6"/>
+      <c r="G87" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" s="5"/>
+      <c r="B88" s="5"/>
+      <c r="C88" s="5"/>
+      <c r="D88" s="5"/>
+      <c r="E88" s="5"/>
+      <c r="F88" s="6"/>
+      <c r="G88" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5"/>
+      <c r="F89" s="6"/>
+      <c r="G89" s="11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="6"/>
+      <c r="G90" s="11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1415,15 +2205,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034E905B39333B74FA95898E771115485" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5aff7705dba03f1ca66de0bba948c32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e484384a-471b-4d38-9bd4-f717a40f978d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a032af748e954b11f4b97a83e204a1c4" ns3:_="">
     <xsd:import namespace="e484384a-471b-4d38-9bd4-f717a40f978d"/>
@@ -1609,31 +2390,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8FE9B93-FBF1-4A06-954E-D242AA736238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1649,4 +2431,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add light/dark mode to the interface
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38C3A086-FF17-4FE8-82A3-FEE89E692334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F44856C-701C-43DE-AF8C-1CBEC7833F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="81">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -279,6 +279,12 @@
   </si>
   <si>
     <t>User clicks contact sales button in the contact drop down at the nav bar and he should be led to a page that gives contact info about the sales team or line qr.</t>
+  </si>
+  <si>
+    <t>AI Chat</t>
+  </si>
+  <si>
+    <t>Download Brochure for each robot</t>
   </si>
 </sst>
 </file>
@@ -1344,7 +1350,9 @@
       <c r="B26" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C26" s="5"/>
+      <c r="C26" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="D26" s="5" t="s">
         <v>73</v>
       </c>
@@ -1358,30 +1366,50 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
+    <row r="27" spans="1:7" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>20</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="F27" s="6"/>
       <c r="G27" s="11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
+    <row r="28" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="5">
+        <v>21</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>80</v>
+      </c>
       <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
+      <c r="D28" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F28" s="6"/>
       <c r="G28" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="5"/>
+      <c r="A29" s="5">
+        <v>22</v>
+      </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>

</xml_diff>

<commit_message>
Switch to Barlow for display and body text
Replace Archivo + Inter with a single Barlow family across the
storefront and admin, simplifying the font token setup to one Latin
face instead of two.

Also normalize CJK compatibility unit glyphs (e.g. ㎡ from mobile
keyboards) to plain "m²" in admin-submitted product text — Barlow has
no glyph for them, so they were silently falling back to a mismatched
font.

Fix full-bleed spec table and enlarge its type

The scroll-expanding spec section wasn't actually reaching full
viewport width: `left-1/2` + `-translate-x-1/2` don't work as an
offset on a sticky element, since `left` there is a scroll
constraint, not a position. Switch to a negative-margin full-bleed
technique, then size up the spec table's text and padding to fill
the extra width.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D00E2D7-C0F3-4162-A291-D7A86D4D4A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{CA0AAC43-7591-423B-8C77-EEBDFB3BFA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-28965" yWindow="615" windowWidth="29130" windowHeight="15810" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="93">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -339,6 +339,12 @@
   </si>
   <si>
     <t>Make the product page to be customizable from the admin panel by the admin. The admin should be able to fully write specification of the product the admin panel with editable content count.</t>
+  </si>
+  <si>
+    <t>Product Card Order Method</t>
+  </si>
+  <si>
+    <t>Add drag and drop method for product card ordering in shop page.</t>
   </si>
 </sst>
 </file>
@@ -1566,13 +1572,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
+    <row r="33" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="5">
+        <v>26</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="6"/>
+      <c r="D33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>92</v>
+      </c>
       <c r="G33" s="11" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Remove Official Partners section from homepage
CEO wants to hold off until specific partner logos are approved;
the component and its copy stay in the codebase to drop back in
once that list is finalized.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{CA0AAC43-7591-423B-8C77-EEBDFB3BFA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A218F1F8-A1D1-49D1-A333-82D645D6E80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28965" yWindow="615" windowWidth="29130" windowHeight="15810" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <sheet name="WebCredentials" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="97">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -345,6 +344,18 @@
   </si>
   <si>
     <t>Add drag and drop method for product card ordering in shop page.</t>
+  </si>
+  <si>
+    <t>Search Engine</t>
+  </si>
+  <si>
+    <t>Should be able to search any products, services, and other sellable items or features that are available on the web.</t>
+  </si>
+  <si>
+    <t>Product customer review section</t>
+  </si>
+  <si>
+    <t>A section where the customers can post reviews on products. Includes start rating, and text reviews.</t>
   </si>
 </sst>
 </file>
@@ -1551,7 +1562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>25</v>
       </c>
@@ -1593,30 +1604,52 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
+    <row r="34" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="5">
+        <v>27</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="6"/>
+      <c r="D34" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>94</v>
+      </c>
       <c r="G34" s="11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
+    <row r="35" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="5">
+        <v>28</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>95</v>
+      </c>
       <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="6"/>
+      <c r="D35" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>96</v>
+      </c>
       <c r="G35" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="5"/>
+      <c r="A36" s="5">
+        <v>29</v>
+      </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -2355,23 +2388,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034E905B39333B74FA95898E771115485" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5aff7705dba03f1ca66de0bba948c32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e484384a-471b-4d38-9bd4-f717a40f978d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a032af748e954b11f4b97a83e204a1c4" ns3:_="">
     <xsd:import namespace="e484384a-471b-4d38-9bd4-f717a40f978d"/>
@@ -2557,10 +2573,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2582,19 +2625,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add Sokochan fulfilment integration (gated, manual send)
Adds an end-to-end 3PL loop, off until Sokochan credentials are set.
Admins push a paid order to the warehouse via a manual "Send to
warehouse" button (carrier chosen at send); Sokochan's shipping webhook
updates fulfilment status + tracking, shown in the admin and to the
customer. New lib/sokochan.ts client, fulfill + webhook routes, an
orders.fulfillment jsonb column, and a per-product warehouse SKU field
(with the same pre-migration graceful degradation as `visible`).
Services are never shipped; missing-SKU lines block the send; the push
is idempotent; the webhook only ever writes fulfilment fields and is
guarded by an optional shared-secret token. EN/TH throughout.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A218F1F8-A1D1-49D1-A333-82D645D6E80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{508B8C99-796D-43CC-B50B-50A532EF02B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-28920" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="WebCredentials" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="98">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -334,9 +335,6 @@
     </r>
   </si>
   <si>
-    <t>Editable product pagetempate</t>
-  </si>
-  <si>
     <t>Make the product page to be customizable from the admin panel by the admin. The admin should be able to fully write specification of the product the admin panel with editable content count.</t>
   </si>
   <si>
@@ -356,6 +354,12 @@
   </si>
   <si>
     <t>A section where the customers can post reviews on products. Includes start rating, and text reviews.</t>
+  </si>
+  <si>
+    <t>Editable product page template</t>
+  </si>
+  <si>
+    <t>Order management dashboard for admin</t>
   </si>
 </sst>
 </file>
@@ -1188,7 +1192,7 @@
         <v>60</v>
       </c>
       <c r="G14" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -1211,7 +1215,7 @@
         <v>60</v>
       </c>
       <c r="G15" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -1257,7 +1261,7 @@
         <v>60</v>
       </c>
       <c r="G17" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="257.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1387,7 +1391,7 @@
         <v>70</v>
       </c>
       <c r="G23" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -1408,7 +1412,7 @@
         <v>74</v>
       </c>
       <c r="G24" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="46" customHeight="1" x14ac:dyDescent="0.35">
@@ -1429,7 +1433,7 @@
         <v>75</v>
       </c>
       <c r="G25" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -1538,7 +1542,7 @@
         <v>86</v>
       </c>
       <c r="G30" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -1562,12 +1566,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>25</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5" t="s">
@@ -1577,10 +1581,10 @@
         <v>27</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G32" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -1588,7 +1592,7 @@
         <v>26</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
@@ -1598,10 +1602,10 @@
         <v>27</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G33" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -1609,7 +1613,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
@@ -1619,10 +1623,10 @@
         <v>24</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G34" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -1630,7 +1634,7 @@
         <v>28</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
@@ -1640,23 +1644,29 @@
         <v>27</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G35" s="11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>29</v>
       </c>
-      <c r="B36" s="5"/>
+      <c r="B36" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
+      <c r="D36" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F36" s="6"/>
       <c r="G36" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -2388,6 +2398,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034E905B39333B74FA95898E771115485" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5aff7705dba03f1ca66de0bba948c32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e484384a-471b-4d38-9bd4-f717a40f978d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a032af748e954b11f4b97a83e204a1c4" ns3:_="">
     <xsd:import namespace="e484384a-471b-4d38-9bd4-f717a40f978d"/>
@@ -2573,37 +2600,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2625,9 +2625,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add robot comparison with AssistiveTouch-style floating launcher (PRD #30)
Customers pick 2-3 robots and see them side by side at /compare: image,
price, quick specs, and features per column, with add-to-cart CTAs.
Selection lives in a persisted site-wide provider; services are never
comparable and stale ids drop out against the live catalog. Entry
points: a draggable floating button that snaps to the screen edge,
dims when idle, and remembers its position (iOS AssistiveTouch
behavior), plus an add-to-comparison toggle on every robot's detail
page. EN/TH throughout; compare URLs are shareable and noindexed.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{508B8C99-796D-43CC-B50B-50A532EF02B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3FB53F1-0B93-48D7-BCD6-AB0445B33A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <sheet name="WebCredentials" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="100">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -360,6 +359,12 @@
   </si>
   <si>
     <t>Order management dashboard for admin</t>
+  </si>
+  <si>
+    <t>Robot Comparison feature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User will see a button or a choice shown on the website, through the button is to choose a robot and another robot for comparison. In addition, if we go to a robot's product details page, there should be a button or something that allows the user to compare that robot with another robot as desire. The robot comparison is minimum 2 robots and maximum 3 robots. </t>
   </si>
 </sst>
 </file>
@@ -1370,7 +1375,7 @@
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.35">
@@ -1566,7 +1571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="68.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>25</v>
       </c>
@@ -1664,18 +1669,27 @@
       <c r="E36" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F36" s="6"/>
       <c r="G36" s="11" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
+    <row r="37" spans="1:7" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="5">
+        <v>30</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="6"/>
+      <c r="D37" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="G37" s="11" t="b">
         <v>0</v>
       </c>
@@ -2398,23 +2412,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034E905B39333B74FA95898E771115485" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5aff7705dba03f1ca66de0bba948c32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e484384a-471b-4d38-9bd4-f717a40f978d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a032af748e954b11f4b97a83e204a1c4" ns3:_="">
     <xsd:import namespace="e484384a-471b-4d38-9bd4-f717a40f978d"/>
@@ -2600,10 +2597,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2625,19 +2649,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Remove Amex from footer payment methods
Amex has limited acceptance and higher merchant fees in Thailand/SEA,
and it isn't confirmed as a method our Omise account will actually
support. Better to only advertise payment methods we're sure we can
take.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3FB53F1-0B93-48D7-BCD6-AB0445B33A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60685BD4-1817-48E1-AC5D-B836537EB769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
@@ -1691,11 +1691,13 @@
         <v>99</v>
       </c>
       <c r="G37" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="5"/>
+      <c r="A38" s="5">
+        <v>31</v>
+      </c>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>

</xml_diff>

<commit_message>
Add metadataBase, sitemap, and robots.txt
Open Graph images had no absolute base, so LINE and Facebook link previews
rendered without an image. Adds canonical and hreflang alternates, a
sitemap covering both locales for static, category, and product pages, and
crawl rules that keep account and checkout routes out of the index.
</commit_message>
<xml_diff>
--- a/docs/PRD-ecommerceRaasPal.xlsx
+++ b/docs/PRD-ecommerceRaasPal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\SoftwareWorkSpace\ecommerce-raaspal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F549AFF9-1A85-4D84-866E-552E3F6870FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DE5544A-2ED9-4460-86E5-6B0D418339E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="3" xr2:uid="{F12EA071-E415-43DC-AFC3-0A64716A9228}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUIREMENTS" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="WebCredentials" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="106">
   <si>
     <t>PROJECT REQUIREMENTS</t>
   </si>
@@ -377,6 +378,12 @@
   </si>
   <si>
     <t>For demo package, the user should not see the demo package recommendation in upselling program since the user already added the robot to the cart and the purpose of demo is to make the user buy the product or add the product to the cart later after demo. If the user enters the demo package's product details page, the user should be asked to choose which robot to demo and also the demo cost should depend on how much the area to demo is.</t>
+  </si>
+  <si>
+    <t>re_FbanmNCc_3SKoFgWoUCtRkKdmocF6REp8</t>
+  </si>
+  <si>
+    <t>Resend - API Key</t>
   </si>
 </sst>
 </file>
@@ -2406,7 +2413,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E048D108-EE43-43FF-98E7-58D5322B5F5D}">
-  <dimension ref="A2:E4"/>
+  <dimension ref="A2:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="13.453125" customWidth="1"/>
@@ -2432,6 +2439,14 @@
       </c>
       <c r="E4" s="8" t="s">
         <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2444,23 +2459,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034E905B39333B74FA95898E771115485" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5aff7705dba03f1ca66de0bba948c32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e484384a-471b-4d38-9bd4-f717a40f978d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a032af748e954b11f4b97a83e204a1c4" ns3:_="">
     <xsd:import namespace="e484384a-471b-4d38-9bd4-f717a40f978d"/>
@@ -2646,31 +2644,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8FE9B93-FBF1-4A06-954E-D242AA736238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="e484384a-471b-4d38-9bd4-f717a40f978d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08118D97-A8F3-495E-81C2-8AE777CE24C3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2686,4 +2677,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD999FCF-7AEA-4702-845A-AD3F14269116}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8FE9B93-FBF1-4A06-954E-D242AA736238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e484384a-471b-4d38-9bd4-f717a40f978d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>